<commit_message>
Change PSO logic a bit
Trying to make it feasible for SQA as well
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -483,30 +483,30 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-37.20769781399783</v>
+        <v>-52.48640960162402</v>
       </c>
       <c r="E2" t="n">
-        <v>1.621526002883911</v>
+        <v>6.943673133850098</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>-37.20769781399783</v>
+        <v>-23.62273046381496</v>
       </c>
       <c r="H2" t="n">
-        <v>-37.20769781399783</v>
+        <v>-23.62273046381496</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>54.99267211624238</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -519,30 +519,30 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>29.30571366171228</v>
+        <v>-52.48640960162402</v>
       </c>
       <c r="E3" t="n">
-        <v>1.467869997024536</v>
+        <v>6.653419017791748</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>42.18649296071128</v>
+        <v>36.74073963915244</v>
       </c>
       <c r="H3" t="n">
-        <v>42.18649296071128</v>
+        <v>36.74073963915244</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>43.95313298862828</v>
+        <v>170.0004818733412</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -555,30 +555,30 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-37.20769781399783</v>
+        <v>-52.48640960162402</v>
       </c>
       <c r="E4" t="n">
-        <v>1.306142330169678</v>
+        <v>5.541934967041016</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>-8.374083115932198</v>
+        <v>215.4021182827348</v>
       </c>
       <c r="H4" t="n">
-        <v>-8.374083115932198</v>
+        <v>215.4021182827348</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>77.49368112535626</v>
+        <v>510.3959861565191</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -591,30 +591,30 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>29.30571366171228</v>
+        <v>-52.48640960162402</v>
       </c>
       <c r="E5" t="n">
-        <v>1.339087009429932</v>
+        <v>5.45050311088562</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>71.73574975413641</v>
+        <v>241.8793328946267</v>
       </c>
       <c r="H5" t="n">
-        <v>71.73574975413641</v>
+        <v>241.8793328946267</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>144.7841761583124</v>
+        <v>560.8418345444276</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -627,30 +627,30 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>-37.20769781399783</v>
+        <v>-52.48640960162402</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4937999248504639</v>
+        <v>1.161741018295288</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>-37.20769781399784</v>
+        <v>2.474372609474241</v>
       </c>
       <c r="H6" t="n">
-        <v>-37.20769781399784</v>
+        <v>2.474372609474241</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.90966594953582e-14</v>
+        <v>104.7143110535754</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -663,22 +663,30 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>29.30571366171228</v>
+        <v>-52.48640960162402</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01910996437072754</v>
+        <v>1.152054786682129</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.995130119093924</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.995130119093924</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>103.8012318507536</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -691,19 +699,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>28.68220582762679</v>
+        <v>-37.20769781399783</v>
       </c>
       <c r="E8" t="n">
-        <v>0.639718770980835</v>
+        <v>1.588465929031372</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>28.68220582762679</v>
+        <v>-37.20769781399783</v>
       </c>
       <c r="H8" t="n">
-        <v>28.68220582762679</v>
+        <v>-37.20769781399783</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -714,7 +722,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -727,30 +735,30 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>50.43461998035004</v>
+        <v>29.30571366171228</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6622488498687744</v>
+        <v>1.501446962356567</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>50.43461998035004</v>
+        <v>43.34401344621553</v>
       </c>
       <c r="H9" t="n">
-        <v>50.43461998035004</v>
+        <v>43.34401344621553</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>47.90294461535058</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -763,30 +771,30 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>28.68220582762679</v>
+        <v>-37.20769781399783</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5462441444396973</v>
+        <v>1.338070869445801</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>28.68220582762679</v>
+        <v>-21.64560616283681</v>
       </c>
       <c r="H10" t="n">
-        <v>28.68220582762679</v>
+        <v>-21.64560616283681</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>41.82492485548632</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -799,30 +807,30 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>50.43461998035004</v>
+        <v>29.30571366171228</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5789539813995361</v>
+        <v>1.272475957870483</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>64.35823551244289</v>
+        <v>46.27201546869094</v>
       </c>
       <c r="H11" t="n">
-        <v>64.35823551244289</v>
+        <v>46.27201546869094</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>27.60725774778846</v>
+        <v>57.89417723392631</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -835,30 +843,30 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>28.68220582762679</v>
+        <v>-37.20769781399783</v>
       </c>
       <c r="E12" t="n">
-        <v>0.476259708404541</v>
+        <v>0.4825079441070557</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>28.6822058276268</v>
+        <v>-37.20769781399784</v>
       </c>
       <c r="H12" t="n">
-        <v>28.6822058276268</v>
+        <v>-37.20769781399784</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>2.47729459871494e-14</v>
+        <v>-1.90966594953582e-14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -871,22 +879,30 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>50.43461998035004</v>
+        <v>29.30571366171228</v>
       </c>
       <c r="E13" t="n">
-        <v>0.01233482360839844</v>
+        <v>0.7112162113189697</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>33.05758801121466</v>
+      </c>
+      <c r="H13" t="n">
+        <v>33.05758801121466</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>12.80253534451265</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -899,30 +915,30 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.1285787260737514</v>
+        <v>33.49034507132686</v>
       </c>
       <c r="E14" t="n">
-        <v>0.200758695602417</v>
+        <v>2.270151138305664</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1285787260737514</v>
+        <v>35.96248888167683</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1285787260737514</v>
+        <v>35.96248888167683</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>7.381661207386374</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -935,30 +951,30 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.1285787260737514</v>
+        <v>49.39427710429008</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1994681358337402</v>
+        <v>2.288674116134644</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1285787260737514</v>
+        <v>68.72877853827845</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1285787260737514</v>
+        <v>68.72877853827845</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>39.14320153560684</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -971,30 +987,30 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.1285787260737514</v>
+        <v>33.49034507132686</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1600308418273926</v>
+        <v>1.883595943450928</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1285787260737514</v>
+        <v>94.76198536502997</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1285787260737514</v>
+        <v>94.76198536502997</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>182.953147133027</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1007,30 +1023,30 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.1285787260737514</v>
+        <v>49.39427710429008</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1647708415985107</v>
+        <v>1.86188006401062</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1285787260737514</v>
+        <v>137.5470950204093</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1285787260737514</v>
+        <v>137.5470950204093</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>178.4676749697038</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1043,30 +1059,30 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.1285787260737514</v>
+        <v>33.49034507132686</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1209521293640137</v>
+        <v>0.6509149074554443</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1285787260737514</v>
+        <v>53.1305200779526</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1285787260737514</v>
+        <v>53.1305200779526</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>58.64428976409947</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1079,30 +1095,30 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.1285787260737514</v>
+        <v>49.39427710429008</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1226701736450195</v>
+        <v>0.9690532684326172</v>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1285787260737514</v>
+        <v>137.6176652130162</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1285787260737514</v>
+        <v>137.6176652130162</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>178.6105461619635</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>5</v>
+        <v>500</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1115,30 +1131,30 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>8.340019847439855</v>
+        <v>-21.09572539323537</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1867198944091797</v>
+        <v>14.03849601745605</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>8.340019847439855</v>
+        <v>203.6001746162661</v>
       </c>
       <c r="H20" t="n">
-        <v>8.340019847439855</v>
+        <v>203.6001746162661</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1065.125260312468</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>5</v>
+        <v>500</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1151,30 +1167,30 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>8.340019847439855</v>
+        <v>82.85450259535968</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1899068355560303</v>
+        <v>13.15287590026855</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>8.340019847439855</v>
+        <v>209.2044521621971</v>
       </c>
       <c r="H21" t="n">
-        <v>8.340019847439855</v>
+        <v>209.2044521621971</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>152.4961777682722</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>5</v>
+        <v>500</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1187,30 +1203,30 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>8.340019847439855</v>
+        <v>-21.09572539323537</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1465179920196533</v>
+        <v>11.83529210090637</v>
       </c>
       <c r="F22" t="n">
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>8.340019847439855</v>
+        <v>394.6920571810572</v>
       </c>
       <c r="H22" t="n">
-        <v>8.340019847439855</v>
+        <v>394.6920571810572</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1970.957503588005</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>5</v>
+        <v>500</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1223,30 +1239,30 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>8.340019847439855</v>
+        <v>82.85450259535968</v>
       </c>
       <c r="E23" t="n">
-        <v>0.1470060348510742</v>
+        <v>11.94407987594604</v>
       </c>
       <c r="F23" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>8.340019847439855</v>
+        <v>18431.91573036496</v>
       </c>
       <c r="H23" t="n">
-        <v>8.340019847439855</v>
+        <v>18431.91573036496</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>22146.12441448323</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>5</v>
+        <v>500</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1259,30 +1275,30 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.340019847439855</v>
+        <v>-21.09572539323537</v>
       </c>
       <c r="E24" t="n">
-        <v>0.09516477584838867</v>
+        <v>1.640885829925537</v>
       </c>
       <c r="F24" t="n">
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>8.340019847439855</v>
+        <v>96.80445656431655</v>
       </c>
       <c r="H24" t="n">
-        <v>8.340019847439855</v>
+        <v>96.80445656431655</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>558.8818576267505</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>5</v>
+        <v>500</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1295,30 +1311,30 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8.340019847439855</v>
+        <v>82.85450259535968</v>
       </c>
       <c r="E25" t="n">
-        <v>0.09894704818725586</v>
+        <v>2.763493061065674</v>
       </c>
       <c r="F25" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>8.340019847439855</v>
+        <v>269.7209089193374</v>
       </c>
       <c r="H25" t="n">
-        <v>8.340019847439855</v>
+        <v>269.7209089193374</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>225.535608169161</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1331,30 +1347,30 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-10.65196883415753</v>
+        <v>-5.177972017787694</v>
       </c>
       <c r="E26" t="n">
-        <v>0.5145070552825928</v>
+        <v>8.216505765914917</v>
       </c>
       <c r="F26" t="n">
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>-10.65196883415753</v>
+        <v>27.37055227426306</v>
       </c>
       <c r="H26" t="n">
-        <v>-10.65196883415753</v>
+        <v>27.37055227426306</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>628.5959866186613</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1367,30 +1383,30 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.06733358914136289</v>
+        <v>12.28666255021365</v>
       </c>
       <c r="E27" t="n">
-        <v>0.3948042392730713</v>
+        <v>7.932331800460815</v>
       </c>
       <c r="F27" t="n">
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>0.06733358914136289</v>
+        <v>128.1952128314461</v>
       </c>
       <c r="H27" t="n">
-        <v>0.06733358914136289</v>
+        <v>128.1952128314461</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>943.3688750507517</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1403,30 +1419,30 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-10.65196883415753</v>
+        <v>-5.177972017787694</v>
       </c>
       <c r="E28" t="n">
-        <v>0.330949068069458</v>
+        <v>6.832162857055664</v>
       </c>
       <c r="F28" t="n">
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>-10.65196883415753</v>
+        <v>154.9072260799256</v>
       </c>
       <c r="H28" t="n">
-        <v>-10.65196883415753</v>
+        <v>154.9072260799256</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>3091.658231210571</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1439,30 +1455,30 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.06733358914136289</v>
+        <v>12.28666255021365</v>
       </c>
       <c r="E29" t="n">
-        <v>0.3350238800048828</v>
+        <v>6.418770790100098</v>
       </c>
       <c r="F29" t="n">
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>0.06733358914136289</v>
+        <v>348.4054571620763</v>
       </c>
       <c r="H29" t="n">
-        <v>0.06733358914136289</v>
+        <v>348.4054571620763</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>2735.639505343281</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1475,54 +1491,1790 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>-10.65196883415753</v>
+        <v>-5.177972017787694</v>
       </c>
       <c r="E30" t="n">
-        <v>0.2301521301269531</v>
+        <v>1.204095840454102</v>
       </c>
       <c r="F30" t="n">
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>-10.65196883415753</v>
+        <v>51.34398742885062</v>
       </c>
       <c r="H30" t="n">
-        <v>-10.65196883415753</v>
+        <v>51.34398742885062</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>1091.584876327461</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
+        <v>350</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>12.28666255021365</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1.924742937088013</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>72.36900826347069</v>
+      </c>
+      <c r="H31" t="n">
+        <v>72.36900826347069</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>489.0046053410354</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>200</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>-44.55700580317149</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3.480612277984619</v>
+      </c>
+      <c r="F32" t="n">
+        <v>100</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-19.76857980968688</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-19.76857980968688</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>55.63306049555111</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>200</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>-31.3058949778858</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3.19782280921936</v>
+      </c>
+      <c r="F33" t="n">
+        <v>100</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-5.491467889805981</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-5.491467889805981</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>82.45867785065687</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>200</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>-44.55700580317149</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2.819736242294312</v>
+      </c>
+      <c r="F34" t="n">
+        <v>100</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-9.511657497837698</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-9.511657497837698</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>78.65283511227167</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>200</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>-31.3058949778858</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2.706088781356812</v>
+      </c>
+      <c r="F35" t="n">
+        <v>100</v>
+      </c>
+      <c r="G35" t="n">
+        <v>27.36449033702085</v>
+      </c>
+      <c r="H35" t="n">
+        <v>27.36449033702085</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>187.4100240748616</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>200</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>-44.55700580317149</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.7892518043518066</v>
+      </c>
+      <c r="F36" t="n">
+        <v>100</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-39.97656184287219</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-39.97656184287219</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>10.27996356068717</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>200</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>-31.3058949778858</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.7973949909210205</v>
+      </c>
+      <c r="F37" t="n">
+        <v>100</v>
+      </c>
+      <c r="G37" t="n">
+        <v>31.58982859856025</v>
+      </c>
+      <c r="H37" t="n">
+        <v>31.58982859856025</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>200.9069653522923</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>50</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>28.68220582762679</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.646129846572876</v>
+      </c>
+      <c r="F38" t="n">
+        <v>100</v>
+      </c>
+      <c r="G38" t="n">
+        <v>28.68220582762679</v>
+      </c>
+      <c r="H38" t="n">
+        <v>28.68220582762679</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>50</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>50.43461998035004</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.7727930545806885</v>
+      </c>
+      <c r="F39" t="n">
+        <v>100</v>
+      </c>
+      <c r="G39" t="n">
+        <v>64.35823551244289</v>
+      </c>
+      <c r="H39" t="n">
+        <v>64.35823551244289</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>27.60725774778846</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>50</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>28.68220582762679</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.5869367122650146</v>
+      </c>
+      <c r="F40" t="n">
+        <v>100</v>
+      </c>
+      <c r="G40" t="n">
+        <v>31.4687279078982</v>
+      </c>
+      <c r="H40" t="n">
+        <v>31.4687279078982</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>9.715159625510477</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>50</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>50.43461998035004</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.5678300857543945</v>
+      </c>
+      <c r="F41" t="n">
+        <v>100</v>
+      </c>
+      <c r="G41" t="n">
+        <v>50.43461998035004</v>
+      </c>
+      <c r="H41" t="n">
+        <v>50.43461998035004</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>50</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>28.68220582762679</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.273831844329834</v>
+      </c>
+      <c r="F42" t="n">
+        <v>100</v>
+      </c>
+      <c r="G42" t="n">
+        <v>28.6822058276268</v>
+      </c>
+      <c r="H42" t="n">
+        <v>28.6822058276268</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2.47729459871494e-14</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>50</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>50.43461998035004</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.2814719676971436</v>
+      </c>
+      <c r="F43" t="n">
+        <v>100</v>
+      </c>
+      <c r="G43" t="n">
+        <v>53.98663432101151</v>
+      </c>
+      <c r="H43" t="n">
+        <v>53.98663432101151</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>7.042809764493876</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>10</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.1845669746398926</v>
+      </c>
+      <c r="F44" t="n">
+        <v>100</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>10</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.1920809745788574</v>
+      </c>
+      <c r="F45" t="n">
+        <v>100</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>10</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.1519408226013184</v>
+      </c>
+      <c r="F46" t="n">
+        <v>100</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>10</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.1553223133087158</v>
+      </c>
+      <c r="F47" t="n">
+        <v>100</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>10</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.12105393409729</v>
+      </c>
+      <c r="F48" t="n">
+        <v>100</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>10</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.1231920719146729</v>
+      </c>
+      <c r="F49" t="n">
+        <v>100</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.1285787260737514</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>450</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>-46.10476965696535</v>
+      </c>
+      <c r="E50" t="n">
+        <v>12.09219813346863</v>
+      </c>
+      <c r="F50" t="n">
+        <v>100</v>
+      </c>
+      <c r="G50" t="n">
+        <v>60.67439585487367</v>
+      </c>
+      <c r="H50" t="n">
+        <v>60.67439585487367</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>231.6011256672815</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>450</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>11.6683923675474</v>
+      </c>
+      <c r="E51" t="n">
+        <v>11.6871931552887</v>
+      </c>
+      <c r="F51" t="n">
+        <v>100</v>
+      </c>
+      <c r="G51" t="n">
+        <v>245.1761157072271</v>
+      </c>
+      <c r="H51" t="n">
+        <v>245.1761157072271</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>2001.198759729068</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>450</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>-46.10476965696535</v>
+      </c>
+      <c r="E52" t="n">
+        <v>9.991870880126953</v>
+      </c>
+      <c r="F52" t="n">
+        <v>100</v>
+      </c>
+      <c r="G52" t="n">
+        <v>206.4918482428754</v>
+      </c>
+      <c r="H52" t="n">
+        <v>206.4918482428754</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>547.8752410634359</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>450</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>11.6683923675474</v>
+      </c>
+      <c r="E53" t="n">
+        <v>9.699477910995483</v>
+      </c>
+      <c r="F53" t="n">
+        <v>100</v>
+      </c>
+      <c r="G53" t="n">
+        <v>607.0914926779016</v>
+      </c>
+      <c r="H53" t="n">
+        <v>607.0914926779016</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>5102.871771490723</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>450</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>-46.10476965696535</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1.694218158721924</v>
+      </c>
+      <c r="F54" t="n">
+        <v>100</v>
+      </c>
+      <c r="G54" t="n">
+        <v>77.42064236671558</v>
+      </c>
+      <c r="H54" t="n">
+        <v>77.42064236671558</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>267.9232820004321</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>450</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>11.6683923675474</v>
+      </c>
+      <c r="E55" t="n">
+        <v>2.421242713928223</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>174.7608391843943</v>
+      </c>
+      <c r="H55" t="n">
+        <v>174.7608391843943</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1397.728510316864</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>400</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>-11.15928385577044</v>
+      </c>
+      <c r="E56" t="n">
+        <v>9.19330883026123</v>
+      </c>
+      <c r="F56" t="n">
+        <v>100</v>
+      </c>
+      <c r="G56" t="n">
+        <v>71.7381937838978</v>
+      </c>
+      <c r="H56" t="n">
+        <v>71.7381937838978</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>742.856609000067</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>400</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>-1.597093151920724</v>
+      </c>
+      <c r="E57" t="n">
+        <v>8.838445901870728</v>
+      </c>
+      <c r="F57" t="n">
+        <v>100</v>
+      </c>
+      <c r="G57" t="n">
+        <v>149.5886999686935</v>
+      </c>
+      <c r="H57" t="n">
+        <v>149.5886999686935</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>9466.310273686446</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>400</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>-11.15928385577044</v>
+      </c>
+      <c r="E58" t="n">
+        <v>8.252639055252075</v>
+      </c>
+      <c r="F58" t="n">
+        <v>100</v>
+      </c>
+      <c r="G58" t="n">
+        <v>312.9965973185054</v>
+      </c>
+      <c r="H58" t="n">
+        <v>312.9965973185054</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>2904.808994590236</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>400</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>-1.597093151920724</v>
+      </c>
+      <c r="E59" t="n">
+        <v>7.780879974365234</v>
+      </c>
+      <c r="F59" t="n">
+        <v>100</v>
+      </c>
+      <c r="G59" t="n">
+        <v>449.816357617023</v>
+      </c>
+      <c r="H59" t="n">
+        <v>449.816357617023</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
+        <v>28264.69140050203</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>400</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>-11.15928385577044</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1.360202074050903</v>
+      </c>
+      <c r="F60" t="n">
+        <v>100</v>
+      </c>
+      <c r="G60" t="n">
+        <v>92.12710234094284</v>
+      </c>
+      <c r="H60" t="n">
+        <v>92.12710234094284</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="n">
+        <v>925.5646467251042</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>400</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>-1.597093151920724</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1.505948066711426</v>
+      </c>
+      <c r="F61" t="n">
+        <v>100</v>
+      </c>
+      <c r="G61" t="n">
+        <v>131.6552064879769</v>
+      </c>
+      <c r="H61" t="n">
+        <v>131.6552064879769</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="n">
+        <v>8343.426899028611</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>5</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.1873164176940918</v>
+      </c>
+      <c r="F62" t="n">
+        <v>100</v>
+      </c>
+      <c r="G62" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="H62" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>5</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.1891829967498779</v>
+      </c>
+      <c r="F63" t="n">
+        <v>100</v>
+      </c>
+      <c r="G63" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="H63" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>5</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.1474730968475342</v>
+      </c>
+      <c r="F64" t="n">
+        <v>100</v>
+      </c>
+      <c r="G64" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="H64" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>5</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.1457369327545166</v>
+      </c>
+      <c r="F65" t="n">
+        <v>100</v>
+      </c>
+      <c r="G65" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="H65" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>5</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.09459900856018066</v>
+      </c>
+      <c r="F66" t="n">
+        <v>100</v>
+      </c>
+      <c r="G66" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="H66" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>5</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.09978890419006348</v>
+      </c>
+      <c r="F67" t="n">
+        <v>100</v>
+      </c>
+      <c r="G67" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="H67" t="n">
+        <v>8.340019847439855</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
         <v>20</v>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>RCSPP</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.3834939002990723</v>
+      </c>
+      <c r="F68" t="n">
+        <v>100</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="H68" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>20</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.3953280448913574</v>
+      </c>
+      <c r="F69" t="n">
+        <v>100</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>20</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.3287570476531982</v>
+      </c>
+      <c r="F70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="H70" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>20</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.3357319831848145</v>
+      </c>
+      <c r="F71" t="n">
+        <v>100</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>20</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
         <is>
           <t>SQA</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D72" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.2358009815216064</v>
+      </c>
+      <c r="F72" t="n">
+        <v>100</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="H72" t="n">
+        <v>-10.65196883415753</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>20</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
         <v>0.06733358914136289</v>
       </c>
-      <c r="E31" t="n">
-        <v>0.003325939178466797</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>0.2354233264923096</v>
+      </c>
+      <c r="F73" t="n">
+        <v>100</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.06733358914136289</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>250</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>27.90417242798865</v>
+      </c>
+      <c r="E74" t="n">
+        <v>4.429360866546631</v>
+      </c>
+      <c r="F74" t="n">
+        <v>100</v>
+      </c>
+      <c r="G74" t="n">
+        <v>56.91461752151878</v>
+      </c>
+      <c r="H74" t="n">
+        <v>56.91461752151878</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
+        <v>103.964542107086</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>250</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>70.51850405979057</v>
+      </c>
+      <c r="E75" t="n">
+        <v>4.516635179519653</v>
+      </c>
+      <c r="F75" t="n">
+        <v>100</v>
+      </c>
+      <c r="G75" t="n">
+        <v>96.66591461092021</v>
+      </c>
+      <c r="H75" t="n">
+        <v>96.66591461092021</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="n">
+        <v>37.07879357304576</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>250</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>27.90417242798865</v>
+      </c>
+      <c r="E76" t="n">
+        <v>3.660101890563965</v>
+      </c>
+      <c r="F76" t="n">
+        <v>100</v>
+      </c>
+      <c r="G76" t="n">
+        <v>122.9498654231892</v>
+      </c>
+      <c r="H76" t="n">
+        <v>122.9498654231892</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="n">
+        <v>340.6146275811682</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>250</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>70.51850405979057</v>
+      </c>
+      <c r="E77" t="n">
+        <v>3.722676992416382</v>
+      </c>
+      <c r="F77" t="n">
+        <v>100</v>
+      </c>
+      <c r="G77" t="n">
+        <v>208.5239455381177</v>
+      </c>
+      <c r="H77" t="n">
+        <v>208.5239455381177</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
+        <v>195.7010338184661</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>250</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SPP</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>27.90417242798865</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.9545090198516846</v>
+      </c>
+      <c r="F78" t="n">
+        <v>100</v>
+      </c>
+      <c r="G78" t="n">
+        <v>56.75281840649112</v>
+      </c>
+      <c r="H78" t="n">
+        <v>56.75281840649112</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="n">
+        <v>103.3847036781011</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>250</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>RCSPP</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>70.51850405979057</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1.566481351852417</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>113.1056823901731</v>
+      </c>
+      <c r="H79" t="n">
+        <v>113.1056823901731</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="n">
+        <v>60.39149425840645</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>